<commit_message>
Taksonomi dan graf berbahasa Indonesia (88 skill, 108 alasan prasyarat); lembar pakar V2 dibuat ulang dari data terbaru
</commit_message>
<xml_diff>
--- a/docs/validasi/V2_pakar_BA.xlsx
+++ b/docs/validasi/V2_pakar_BA.xlsx
@@ -452,7 +452,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Validasi pakar untuk peran Business Analyst, pakar: BA</t>
+          <t>Validasi pakar untuk peran Business Analyst, pakar: pakar_baru</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1355,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>ESCO: 'translate requirement concepts into visual design'.</t>
+          <t>ESCO: 'menerjemahkan konsep kebutuhan menjadi desain visual'.</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr"/>
@@ -1473,17 +1473,17 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Programming fundamentals &amp; OOP</t>
+          <t>Dasar pemrograman &amp; OOP</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>REST API design &amp; development</t>
+          <t>Desain &amp; pengembangan REST API</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Building APIs needs working code in some language.</t>
+          <t>Membangun API membutuhkan kode yang berjalan dalam suatu bahasa.</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr"/>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Python programming</t>
+          <t>Pemrograman Python</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>pandas and NumPy are Python libraries.</t>
+          <t>pandas dan NumPy adalah pustaka Python.</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr"/>
@@ -1537,7 +1537,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Test design &amp; test cases</t>
+          <t>Desain tes &amp; kasus uji</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>UAT scripts are built from test design techniques.</t>
+          <t>Skrip UAT disusun dari teknik desain tes.</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr"/>
@@ -1749,7 +1749,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>70%</t>
+          <t>57%</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr"/>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>48%</t>
+          <t>47%</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr"/>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>41%</t>
+          <t>39%</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr"/>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>36%</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr"/>
@@ -1837,7 +1837,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr"/>
@@ -1893,17 +1893,17 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>erp_crm</t>
+          <t>excel</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Sistem ERP &amp; CRM</t>
+          <t>Microsoft Excel &amp; Spreadsheet</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr"/>
@@ -1915,17 +1915,17 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>excel</t>
+          <t>erp_crm</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Microsoft Excel &amp; Spreadsheet</t>
+          <t>Sistem ERP &amp; CRM</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>21%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr"/>
@@ -1937,17 +1937,17 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>system_modeling_uml</t>
+          <t>jira_confluence</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Pemodelan Sistem (UML/Use Case)</t>
+          <t>Jira/Confluence &amp; Alat Kolaborasi</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>17%</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr"/>
@@ -1969,7 +1969,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>14%</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr"/>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>14%</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr"/>
@@ -2003,12 +2003,12 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>data_analysis</t>
+          <t>system_modeling_uml</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Analisis Data</t>
+          <t>Pemodelan Sistem (UML/Use Case)</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -2025,12 +2025,12 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>jira_confluence</t>
+          <t>data_analysis</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Jira/Confluence &amp; Alat Kolaborasi</t>
+          <t>Analisis Data</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -2052,12 +2052,12 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>REST API design &amp; development</t>
+          <t>Desain &amp; pengembangan REST API</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>9%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr"/>
@@ -2069,17 +2069,17 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>kpi_metrics</t>
+          <t>data_cleaning</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Metrik &amp; KPI Bisnis</t>
+          <t>Persiapan &amp; Kualitas Data</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>9%</t>
+          <t>7%</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr"/>
@@ -2091,17 +2091,17 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>data_cleaning</t>
+          <t>dashboard_reporting</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Persiapan &amp; Kualitas Data</t>
+          <t>Pelaporan &amp; Dashboard BI</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>7%</t>
+          <t>6%</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr"/>
@@ -2113,17 +2113,17 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>dashboard_reporting</t>
+          <t>kpi_metrics</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Pelaporan &amp; Dashboard BI</t>
+          <t>Metrik &amp; KPI Bisnis</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>6%</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr"/>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr"/>
@@ -2167,7 +2167,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr"/>
@@ -2290,7 +2290,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Authentication &amp; application security</t>
+          <t>Autentikasi &amp; keamanan aplikasi</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Caching &amp; message queues</t>
+          <t>Caching &amp; message queue</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Data structures &amp; algorithms</t>
+          <t>Struktur data &amp; algoritma</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Go back-end</t>
+          <t>Back-end Go</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Node.js back-end</t>
+          <t>Back-end Node.js</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NoSQL databases</t>
+          <t>Database NoSQL</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2460,7 +2460,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Programming fundamentals &amp; OOP</t>
+          <t>Dasar pemrograman &amp; OOP</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Python back-end (Django, FastAPI, Flask)</t>
+          <t>Back-end Python (Django, FastAPI, Flask)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2494,7 +2494,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Python programming</t>
+          <t>Pemrograman Python</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>REST API design &amp; development</t>
+          <t>Desain &amp; pengembangan REST API</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>System design &amp; microservices</t>
+          <t>Desain sistem &amp; microservice</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Big data processing (Spark &amp; Hadoop)</t>
+          <t>Pemrosesan big data (Spark &amp; Hadoop)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Data warehousing &amp; modelling</t>
+          <t>Data warehouse &amp; pemodelan</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2987,7 +2987,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ETL / ELT pipelines</t>
+          <t>Pipeline ETL / ELT</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Streaming data (Kafka)</t>
+          <t>Data streaming (Kafka)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3021,7 +3021,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Workflow orchestration (Airflow)</t>
+          <t>Orkestrasi alur kerja (Airflow)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3072,7 +3072,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Math &amp; statistics for machine learning</t>
+          <t>Matematika &amp; statistika untuk machine learning</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3089,7 +3089,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Model deployment &amp; MLOps</t>
+          <t>Deployment model &amp; MLOps</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Accessible design (WCAG)</t>
+          <t>Desain yang mudah diakses (WCAG)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Design systems</t>
+          <t>Design system</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -3157,7 +3157,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Figma &amp; design tools</t>
+          <t>Figma &amp; alat desain</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3174,7 +3174,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Information architecture</t>
+          <t>Arsitektur informasi</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3191,7 +3191,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Prototyping &amp; interaction design</t>
+          <t>Prototyping &amp; desain interaksi</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Usability testing</t>
+          <t>Pengujian usability</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3225,7 +3225,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>User research</t>
+          <t>Riset pengguna</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3242,7 +3242,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Visual design fundamentals</t>
+          <t>Dasar desain visual</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3276,7 +3276,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>CI/CD pipelines</t>
+          <t>Pipeline CI/CD</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Docker &amp; containers</t>
+          <t>Docker &amp; container</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3395,7 +3395,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Monitoring &amp; observability</t>
+          <t>Pemantauan &amp; observability</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3412,7 +3412,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Networking fundamentals</t>
+          <t>Dasar jaringan komputer</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Web servers &amp; reverse proxies</t>
+          <t>Web server &amp; reverse proxy</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3446,7 +3446,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Accounting fundamentals (PSAK)</t>
+          <t>Dasar akuntansi (PSAK)</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3463,7 +3463,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Accounting &amp; ERP software</t>
+          <t>Perangkat lunak akuntansi &amp; ERP</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3480,7 +3480,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Payables, receivables &amp; reconciliation</t>
+          <t>Hutang, piutang &amp; rekonsiliasi</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3497,7 +3497,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Audit &amp; internal control</t>
+          <t>Audit &amp; pengendalian internal</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Budgeting &amp; forecasting</t>
+          <t>Penganggaran &amp; forecasting</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3531,7 +3531,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Cost accounting &amp; inventory</t>
+          <t>Akuntansi biaya &amp; persediaan</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3565,7 +3565,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Financial statements &amp; reporting</t>
+          <t>Laporan keuangan &amp; pelaporan</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3582,7 +3582,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Indonesian tax compliance</t>
+          <t>Kepatuhan pajak Indonesia</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3701,7 +3701,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Content production tools</t>
+          <t>Alat produksi konten</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Conversion optimisation &amp; experiments</t>
+          <t>Optimasi konversi &amp; eksperimen</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -3735,7 +3735,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Email &amp; marketing automation</t>
+          <t>Email &amp; otomasi pemasaran</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -3752,7 +3752,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Marketplace &amp; e-commerce marketing</t>
+          <t>Pemasaran marketplace &amp; e-commerce</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -3769,7 +3769,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Search advertising (Google Ads)</t>
+          <t>Iklan pencarian (Google Ads)</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Social media advertising</t>
+          <t>Iklan media sosial</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -3820,7 +3820,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Web &amp; marketing analytics</t>
+          <t>Analitik web &amp; pemasaran</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -3888,7 +3888,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Mobile back-end services (Firebase &amp; APIs)</t>
+          <t>Layanan back-end mobile (Firebase &amp; API)</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -3905,7 +3905,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>App release &amp; mobile quality</t>
+          <t>Rilis aplikasi &amp; kualitas mobile</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -4041,7 +4041,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Cloud &amp; application security</t>
+          <t>Keamanan cloud &amp; aplikasi</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -4058,7 +4058,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Cryptography fundamentals</t>
+          <t>Dasar kriptografi</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -4075,7 +4075,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Incident response &amp; digital forensics</t>
+          <t>Respons insiden &amp; forensik digital</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -4092,7 +4092,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Network security</t>
+          <t>Keamanan jaringan</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -4126,7 +4126,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Security frameworks &amp; compliance</t>
+          <t>Kerangka keamanan &amp; kepatuhan</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -4143,7 +4143,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>SIEM &amp; security monitoring</t>
+          <t>SIEM &amp; pemantauan keamanan</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -4160,7 +4160,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Vulnerability assessment</t>
+          <t>Penilaian kerentanan</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -4313,7 +4313,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>API testing</t>
+          <t>Pengujian API</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -4330,7 +4330,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Testing in CI/CD</t>
+          <t>Pengujian di CI/CD</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -4347,7 +4347,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Performance &amp; load testing</t>
+          <t>Tes performa &amp; beban</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Web test automation</t>
+          <t>Otomasi tes web</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -4381,7 +4381,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Test design &amp; test cases</t>
+          <t>Desain tes &amp; kasus uji</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Vue, Angular &amp; other frameworks</t>
+          <t>Vue, Angular &amp; framework lain</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -4449,7 +4449,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Front-end testing</t>
+          <t>Pengujian front-end</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -4517,7 +4517,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Responsive &amp; accessible web design</t>
+          <t>Desain web responsif &amp; mudah diakses</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -4551,7 +4551,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Web performance</t>
+          <t>Performa web</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">

</xml_diff>